<commit_message>
added ads to requirements
</commit_message>
<xml_diff>
--- a/tailoringexpert-poi/src/test/resources/basecatalog.xlsx
+++ b/tailoringexpert-poi/src/test/resources/basecatalog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micrf\entwicklung\micrf\git\tailoringexpert\platform\tailoringexpert-poi\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\baed_mi\entwicklung\baed_mi\git\tailoringexpert\platform\tailoringexpert-poi\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C2C21D0-8933-42BE-A79D-E73A9F7F6DA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D2488DC-19D2-49CC-811D-24D7C43529E9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="LOGO" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'8.2.1'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'8.2.1'!$C$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">DRD!$A$1:$D$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">LOGO!$A$1:$B$1</definedName>
   </definedNames>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23379" uniqueCount="3702">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22853" uniqueCount="3400">
   <si>
     <t>1</t>
   </si>
@@ -10551,961 +10551,17 @@
     <t>Rev.1</t>
   </si>
   <si>
-    <t>ECSS-S-ST-00</t>
-  </si>
-  <si>
-    <t>Description, implementation and general requirements (31 July 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-E-ST-10-01</t>
-  </si>
-  <si>
-    <t>System Engineering general requirements (15 February 2017)</t>
-  </si>
-  <si>
-    <t>ECSS-E-ST-10-02</t>
-  </si>
-  <si>
-    <t>Rev.2</t>
-  </si>
-  <si>
-    <t>Verification (1 February 2009)</t>
-  </si>
-  <si>
-    <t>ECSS-E-ST-10-03</t>
-  </si>
-  <si>
-    <t>Testing (1 June 2012)</t>
-  </si>
-  <si>
-    <t>ECSS-E-ST-10-12</t>
-  </si>
-  <si>
-    <t>Methods for the calculation of radiation received and its effects, and a policy for design margins (15 November 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-E-ST-20</t>
-  </si>
-  <si>
-    <t>Electrical and electronic (31 July 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-E-ST-31</t>
-  </si>
-  <si>
-    <t>Thermal control general requirements (15 November 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-E-ST-32</t>
-  </si>
-  <si>
-    <t>Structural general requirements (15 November 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-E-ST-32-01</t>
-  </si>
-  <si>
-    <t>Fracture Control (6 March 2009)</t>
-  </si>
-  <si>
-    <t>ECSS-E-ST-32-10</t>
-  </si>
-  <si>
-    <t>Rev.2 Corr.1</t>
-  </si>
-  <si>
-    <t>Structural factors of safety for spaceflight hardware (01 August 2019)</t>
-  </si>
-  <si>
-    <t>ECSS-E-ST-40</t>
-  </si>
-  <si>
-    <t>Software general requirements (6 March 2009)</t>
-  </si>
-  <si>
-    <t>ECSS-E-ST-50-05</t>
-  </si>
-  <si>
-    <t>Radio frequency and modulation (4 October 2011)</t>
-  </si>
-  <si>
-    <t>ECSS-E-ST-50-14</t>
-  </si>
-  <si>
-    <t>Spacecraft discrete interfaces (31 July 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-M-ST-10</t>
-  </si>
-  <si>
-    <t>Project Planning and Implementation (6 March 2009)</t>
-  </si>
-  <si>
-    <t>ECSS-M-ST-40</t>
-  </si>
-  <si>
-    <t>Configuration and Information Management (6 March 2009)</t>
-  </si>
-  <si>
-    <t>ECSS-M-ST-80</t>
-  </si>
-  <si>
-    <t>Risk Management (31 July 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-10-04</t>
-  </si>
-  <si>
-    <t>CI Control (31 July 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-10-09</t>
-  </si>
-  <si>
-    <t>Nonconformance Control System (1 March 2018)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-20</t>
-  </si>
-  <si>
-    <t>Quality assurance (1 February 2018)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-30</t>
-  </si>
-  <si>
-    <t>Dependability (15 February 2017)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-30-02</t>
-  </si>
-  <si>
-    <t>Failure modes, effects (and criticality) analysis (FMEA/FMECA) (6 March 2009)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-30-09</t>
-  </si>
-  <si>
-    <t>Availability analysis (31 July 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-30-11</t>
-  </si>
-  <si>
-    <t>Derating - EEE components (4 October 2011)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-40</t>
-  </si>
-  <si>
-    <t>Safety (15 February 2017)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-40-12</t>
-  </si>
-  <si>
-    <t>Fault Tree Analysis (31 July 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-60-02</t>
-  </si>
-  <si>
-    <t>ASIC and FPGA development (31 July 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-60-05</t>
-  </si>
-  <si>
-    <t>Generic Procurement Requirements for Hybrids (6 March 2009)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-60-12</t>
-  </si>
-  <si>
-    <t>Design, selection, procurement and use of die form monolithic microwave integrated circuits (MMICs) (31 July 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-60-13</t>
-  </si>
-  <si>
-    <t>Commercial EEE components (21 October 2013)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-60-14</t>
-  </si>
-  <si>
-    <t>Relifing procedure - EEE (15 November 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-60-15</t>
-  </si>
-  <si>
-    <t>Radiation hardness assurance - EEE components (1 October 2012)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70</t>
-  </si>
-  <si>
-    <t>Materials, mechanical parts and processes (15 October 2014)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-01</t>
-  </si>
-  <si>
-    <t>Contamination and Cleanliness Control (15 November 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-02</t>
-  </si>
-  <si>
-    <t>Thermal Vacuum out-gassing Test for the Screening of space materials (15 November 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-04</t>
-  </si>
-  <si>
-    <t>Thermal testing for the evaluation of space materials, processes, mechanical parts and assemblies (15 November 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-07</t>
-  </si>
-  <si>
-    <t>Verification and Approval of Automatic Machine Wave Soldering (16 April 2010)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-08</t>
-  </si>
-  <si>
-    <t>Manual soldering of high- reliability electrical connections (6 March 2009)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-09</t>
-  </si>
-  <si>
-    <t>Measurements of thermo-optical properties of thermal control materials (31 July 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-10</t>
-  </si>
-  <si>
-    <t>Qualification of printed circuit boards (15 November 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-11</t>
-  </si>
-  <si>
-    <t>Procurement of printed circuit boards (15 November 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-18</t>
-  </si>
-  <si>
-    <t>Preparation, assembly and mounting of RF coaxial cables (15 November 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-21</t>
-  </si>
-  <si>
-    <t>Flammability testing for the screening of space materials (5 February 2010)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-22</t>
-  </si>
-  <si>
-    <t>Control of limited shelf-life materials (31 July 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-26</t>
-  </si>
-  <si>
-    <t>Crimping of high-reliability electrical connections (15 March 2017) + correction 1 (1 June 2017)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-28</t>
-  </si>
-  <si>
-    <t>Repair and modification of printed circuit board assemblies for space use (31 July 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-29</t>
-  </si>
-  <si>
-    <t>Determination of offgassing products from materials and assembled articles to be used in a manned space vehicle crew compartment (15 November 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-30</t>
-  </si>
-  <si>
-    <t>Wire wrapping of high-reliability electrical connections (31 July 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-36</t>
-  </si>
-  <si>
-    <t>Material selection for controlling stress-corrosion cracking (6 March 2009)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-38</t>
-  </si>
-  <si>
-    <t>Rev.1 Corrigendum 1</t>
-  </si>
-  <si>
-    <t>High-reliability soldering for surface-mount and mixed technology (15 September 2017)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-39</t>
-  </si>
-  <si>
-    <t>Welding of metallic materials for flight hardware (1 May 2015)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-53</t>
-  </si>
-  <si>
-    <t>Materials and hardware compatibility test for sterilization processes (15 November 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-55</t>
-  </si>
-  <si>
-    <t>Microbial examination of flight hardware and cleanrooms (15 November 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-56</t>
-  </si>
-  <si>
-    <t>Vapour phase bioburden reduction for flight hardware (30 August 2013)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-57</t>
-  </si>
-  <si>
-    <t>Dry heat bioburden reduction for flight hardware (30 August 2013)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-58</t>
-  </si>
-  <si>
-    <t>Bioburden control of cleanrooms (15 November 2008)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-60</t>
-  </si>
-  <si>
-    <t>Corrigendum 1</t>
-  </si>
-  <si>
-    <t>Qualification and procurement of printed circuit boards (1 March 2019)</t>
-  </si>
-  <si>
-    <t>ECSS-Q-ST-70-71</t>
-  </si>
-  <si>
-    <t>Materials, processes and their data selection (15 October 2014)</t>
-  </si>
-  <si>
     <t>Software product assurance (15 February 2017)</t>
   </si>
   <si>
-    <t>ANSI / IPC-A-600</t>
-  </si>
-  <si>
-    <t>Acceptability of Printed Boards</t>
-  </si>
-  <si>
-    <t>ANSI / IPC-A-610</t>
-  </si>
-  <si>
-    <t>Acceptability of Electronic Assemblies</t>
-  </si>
-  <si>
-    <t>ANSI/ESD S20.20- 2014</t>
-  </si>
-  <si>
-    <t>ESD Association Standard for the Development of an Electrostatic Discharge Control Program for Protection of Electrical and Electronic Parts, Assemblies and Equipment (Excluding Electrically Initiated Explosive Devices) (September 2014)</t>
-  </si>
-  <si>
-    <t>CECC 00200</t>
-  </si>
-  <si>
-    <t>Cenelec - QPL</t>
-  </si>
-  <si>
-    <t>CECC MUAHAG PPL</t>
-  </si>
-  <si>
-    <t>Cenelec - PPL (Military User and Ad-Hoc Advisory Group)</t>
-  </si>
-  <si>
-    <t>COL-RIBRE-TN-
-1332</t>
-  </si>
-  <si>
-    <t>Issue 01</t>
-  </si>
-  <si>
-    <t>Fungus growth implementation approach - Technical Note (December 1997)</t>
-  </si>
-  <si>
-    <t>CSG-NT-SBU-166-
-CNES</t>
-  </si>
-  <si>
-    <t>CSG Safety Regulations CNES PSH, Doc. CSG-NT-SBU- 166-CNES, Ed/Rev 01/01, 6 May 2015</t>
-  </si>
-  <si>
-    <t>DIN EN 60812:2006- 11 (IEC 60812:2006)</t>
-  </si>
-  <si>
-    <t>Analysis techniques for system reliability - Procedure for failure mode and effects analysis (FMEA) (IEC 60812: 2006); German version EN 60812:2006</t>
-  </si>
-  <si>
-    <t>EEE-INST-002</t>
-  </si>
-  <si>
-    <t>nstructions for EEE Parts selection, screening, Qualification, and Derating (April 2008)</t>
-  </si>
-  <si>
-    <t>EHB 0004</t>
-  </si>
-  <si>
-    <t>Eurockot Safety Handbook for Launch Service by Eurockot and Khrunichev</t>
-  </si>
-  <si>
-    <t>EN 61340-5.1</t>
-  </si>
-  <si>
-    <t>Electrostatics - Part 5-1: Protection of electronic devices from electrostatic phenomena - General requirements (IEC 61340-5-1:2016); German version EN 61340-5-1: 2016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FprEN 9100:2016 </t>
-  </si>
-  <si>
-    <t>Quality Management Systems - Requirements for Aviation, Space and Defence Organizations; English
-version FprEN 9100:2016</t>
-  </si>
-  <si>
-    <t>EPPL part 1 and
-part 2</t>
-  </si>
-  <si>
-    <t>European PPL</t>
-  </si>
-  <si>
-    <t>ESA/SCC QPL</t>
-  </si>
-  <si>
-    <t>Qualified Parts List</t>
-  </si>
-  <si>
-    <t>ESA-HRE-IPL-RQ-
-0002</t>
-  </si>
-  <si>
-    <t>Issue 1</t>
-  </si>
-  <si>
-    <t>Product Assurance and Safety Requirements for ISS Pressurized Payloads</t>
-  </si>
-  <si>
-    <t>ESCC 20200</t>
-  </si>
-  <si>
-    <t>Component manufacturer evaluation</t>
-  </si>
-  <si>
-    <t>ESCC 20600</t>
-  </si>
-  <si>
-    <t>Preservation, Packaging and dispatch of SCC Electronic Components</t>
-  </si>
-  <si>
-    <t>ESCC 22800</t>
-  </si>
-  <si>
-    <t>ESCC: ESA/SCC Non-conformance Control System</t>
-  </si>
-  <si>
-    <t>ESCC 22900</t>
-  </si>
-  <si>
-    <t>Total Dose Steady-State Irradiation Test Method</t>
-  </si>
-  <si>
-    <t>ESCC 24900</t>
-  </si>
-  <si>
-    <t>Minimum requirements for controlling environmental contamination of components</t>
-  </si>
-  <si>
-    <t>ESCC 25100</t>
-  </si>
-  <si>
-    <t>SEEs Test Method and Guidelines</t>
-  </si>
-  <si>
-    <t>ESCC 25500</t>
-  </si>
-  <si>
-    <t>Methodology for the detection of pure tin in the external surface finish of case and leads of EEE components (April 2013)</t>
-  </si>
-  <si>
-    <t>ESCC 9000</t>
-  </si>
-  <si>
-    <t>Generic Specification Integrated Circuits, Monolithic, Hermetically Sealed</t>
-  </si>
-  <si>
-    <t>GEIA-STD-0005-02</t>
-  </si>
-  <si>
-    <t>Rev. A</t>
-  </si>
-  <si>
-    <t>Standard for Mitigating the Effects of Tin Whiskers in Aerospace and High Performance Electronic Systems (May 2012)</t>
-  </si>
-  <si>
-    <t>IEC 61025</t>
-  </si>
-  <si>
-    <t>Störungsbaum-Analyse</t>
-  </si>
-  <si>
-    <t>IEEE Standard 1149.1</t>
-  </si>
-  <si>
-    <t>Standard Test Access Port and Boundary Scan Architecture</t>
-  </si>
-  <si>
-    <t>IPC/JEDEC 7095</t>
-  </si>
-  <si>
-    <t>Design and Assembly Process Implementation for BGAs</t>
-  </si>
-  <si>
-    <t>IPC/JEDEC J-STD- 033</t>
-  </si>
-  <si>
-    <t>Standard for Handling, Packing, Shipping and Use of Moisture/ reflow Sensitive Surface Mount Devices</t>
-  </si>
-  <si>
-    <t>IPC-TM650 - 2.6.26</t>
-  </si>
-  <si>
-    <t>DC Current Induced Thermal Cycling Test (IPC TEST
-METHODS MANUAL)</t>
-  </si>
-  <si>
-    <t>Space systems - Unmanned spacecraft - Estimating the
-mass of remaining usable propellant</t>
-  </si>
-  <si>
-    <t>ISO 24113:2011</t>
-  </si>
-  <si>
-    <t>ISO 23339:2010-12</t>
-  </si>
-  <si>
-    <t>Space systems - Space debris mitigation requirements (May 2011)</t>
-  </si>
-  <si>
-    <t>ISO 26872:2019</t>
-  </si>
-  <si>
-    <t>Space systems - Disposal of satellites operating at geosynchronous altitude</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ISO 27852:2016-07 </t>
-  </si>
-  <si>
-    <t>Space systems - Estimation of orbit lifetime</t>
-  </si>
-  <si>
-    <t>ISO 9001:2015</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ISO/IEC 25010:2011 </t>
-  </si>
-  <si>
-    <t>Quality management systems - Requirements
-(November 2015)</t>
-  </si>
-  <si>
-    <t>Software-Engineering - Qualitätskriterien und
-Bewertung von Softwareprodukten (SQuaRE) -
-Qualitätsmodell und Leitlinien (March 2011)</t>
-  </si>
-  <si>
-    <t>J-STD-046</t>
-  </si>
-  <si>
-    <t>J-STD-048</t>
-  </si>
-  <si>
-    <t>Notification Standard for Product Discontinuance</t>
-  </si>
-  <si>
-    <t>JEDEC JESD57</t>
-  </si>
-  <si>
-    <t>Test procedure for the management of SINGLE-EVENTEFFECTS in semiconductor devices from heavy ion irradiation</t>
-  </si>
-  <si>
-    <t>KNPR 8715.3
-chapter 20</t>
-  </si>
-  <si>
-    <t>ASA KSC Payload &amp; Cargo Ground Safety Requirements</t>
-  </si>
-  <si>
-    <t>NPR 8715.6B</t>
-  </si>
-  <si>
-    <t>NASA Procedural Requirements for Limiting Orbital Debris and Evaluating the Meteoroid and Orbital Debris Environments</t>
-  </si>
-  <si>
-    <t>MIL QML</t>
-  </si>
-  <si>
-    <t>Military Qualified Manufacture List</t>
-  </si>
-  <si>
-    <t>MIL QPL</t>
-  </si>
-  <si>
-    <t>Military Qualified Product List</t>
-  </si>
-  <si>
-    <t>MIL-HDBK-217F</t>
-  </si>
-  <si>
-    <t>Reliability Prediction of Electronic Equipment (use as Guideline)</t>
-  </si>
-  <si>
-    <t>MIL-PRF-19500</t>
-  </si>
-  <si>
-    <t>Semiconductor Devices; General Specification for</t>
-  </si>
-  <si>
-    <t>MIL-PRF-38534</t>
-  </si>
-  <si>
-    <t>Hybrid Microcircuits, General Specification for</t>
-  </si>
-  <si>
-    <t>MIL-PRF-38535</t>
-  </si>
-  <si>
-    <t>Integrated Circuits (Microcircuits) Manufacturing;
-General Specification for</t>
-  </si>
-  <si>
-    <t>MIL-STD-750</t>
-  </si>
-  <si>
-    <t>Test Method Standard for Semiconductor Devices</t>
-  </si>
-  <si>
-    <t>MIL-STD-810G</t>
-  </si>
-  <si>
-    <t>Test method standard (January 2000)</t>
-  </si>
-  <si>
-    <t>MSFC-HDBK-527</t>
-  </si>
-  <si>
-    <t>Materials Selection Guide for MSFC Spacelab</t>
-  </si>
-  <si>
-    <t>MSFC-STD-3012</t>
-  </si>
-  <si>
-    <t>Electrical, electronic, and electromechanical (EEE) parts
-management and control requirements for MSFC
-space flight hardware (February 2012)</t>
-  </si>
-  <si>
-    <t>MSFC-STD-3029</t>
-  </si>
-  <si>
-    <t>Guidelines for the selection of metallic materials for
-stress corrosion cracking resistance in sodiumchloride environments (February 2005)</t>
-  </si>
-  <si>
-    <t>NASA-GB-8719.13</t>
-  </si>
-  <si>
-    <t>NASA Software Safety Guidebook</t>
-  </si>
-  <si>
-    <t>NASA-STD-6001</t>
-  </si>
-  <si>
-    <t>Flammability, Odour and Offgassing, and Compatibility Requirements and Test Procedures for Materials in Environments that Support Combustion</t>
-  </si>
-  <si>
-    <t>NASA-STD-6004</t>
-  </si>
-  <si>
-    <t>NASA-STD-6016</t>
-  </si>
-  <si>
-    <t>Standard materials and processes requirements for spacecraft</t>
-  </si>
-  <si>
-    <t>Design Criteria for Controlling Stress Corrosion Based
-on Accelerated Testing in Aqueous NaCl Environments
-(as guideline only)</t>
-  </si>
-  <si>
-    <t>NPSL</t>
-  </si>
-  <si>
-    <t>NASA Parts Selection List</t>
-  </si>
-  <si>
-    <t>Space Forces Requirements of Cosmodrom</t>
-  </si>
-  <si>
-    <t>SSP 30233</t>
-  </si>
-  <si>
-    <t>Rev. F</t>
-  </si>
-  <si>
-    <t>Space Station Requirements for Materials and
-Processes (March 1998)</t>
-  </si>
-  <si>
-    <t>SSP 30599</t>
-  </si>
-  <si>
-    <t>Safety review process (February 2015)</t>
-  </si>
-  <si>
-    <t>SSP 41163H</t>
-  </si>
-  <si>
-    <t>Russian Segment Specification (October 2001)</t>
-  </si>
-  <si>
-    <t>SSP 50005</t>
-  </si>
-  <si>
-    <t>Rev. E</t>
-  </si>
-  <si>
-    <t>Flight Crew Integration Standard (NASA−STD−3000/T)
-(June 2006)</t>
-  </si>
-  <si>
-    <t>SSP 50038</t>
-  </si>
-  <si>
-    <t>Rev. B</t>
-  </si>
-  <si>
-    <t>Computer-Based Control System Safety Requirements
-(November 1995)</t>
-  </si>
-  <si>
-    <t>SSP 50094</t>
-  </si>
-  <si>
-    <t>NASA/RSA Joint Specifications Standards Document for
-the Russian Segment (June 2009)</t>
-  </si>
-  <si>
-    <t>SSP 50146</t>
-  </si>
-  <si>
-    <t>NASA/RSA Bilateral S&amp;MA Process Requirements for
-ISS (March 2004)</t>
-  </si>
-  <si>
-    <t>SSP 50260</t>
-  </si>
-  <si>
-    <t>Rev. C</t>
-  </si>
-  <si>
-    <t>International Space Station Medical Operations
-Requirements Document (ISS MORD) (February 2006)</t>
-  </si>
-  <si>
-    <t>SSP 52005</t>
-  </si>
-  <si>
-    <t>Revision F</t>
-  </si>
-  <si>
-    <t>Payload Flight Equipment
-Requirements and Guidelines
-for Safety-Critical Structures
-(August 2014)</t>
-  </si>
-  <si>
-    <t>SSP 51721</t>
-  </si>
-  <si>
-    <t>Baseline DCN 004</t>
-  </si>
-  <si>
-    <t>Payload Safety Policy and Requirements for the
-International Space Station, DCN 004 (09-February-
-2016)</t>
-  </si>
-  <si>
-    <t>UTE C80-810</t>
-  </si>
-  <si>
-    <t>Reliability Data Handbook</t>
-  </si>
-  <si>
-    <t>ATV/HTV/KSC Form 100</t>
-  </si>
-  <si>
-    <t>Integrated Safety Checklist for ISS Cargo At Launch or
-Processing Sites (ATV/HTV/KSC Form 100)</t>
-  </si>
-  <si>
-    <t>Forms for Safety Authorities</t>
-  </si>
-  <si>
-    <t>Launcher organisation requirements defining the launch safety and verification requirements and the technical and operational interfaces to the
-launch system shall be considered.</t>
-  </si>
-  <si>
-    <t>ISS_CM_031</t>
-  </si>
-  <si>
-    <t>Safety Noncompliance Report</t>
-  </si>
-  <si>
-    <t>ISS_EP_03</t>
-  </si>
-  <si>
-    <t>EP5 Battery Design Evaluation Form</t>
-  </si>
-  <si>
-    <t>ISS_OE_622</t>
-  </si>
-  <si>
-    <t>Series and Reflown Equipment Safety Assessment
-Reporting Sheet</t>
-  </si>
-  <si>
-    <t>ISS_OE_764</t>
-  </si>
-  <si>
-    <t>Safety Verification Tracking Log</t>
-  </si>
-  <si>
-    <t>ISS_OE_906</t>
-  </si>
-  <si>
-    <t>Flight Safety Certification</t>
-  </si>
-  <si>
-    <t>ISS_OE_907</t>
-  </si>
-  <si>
-    <t>Multilateral Category 1 Constraints</t>
-  </si>
-  <si>
-    <t>JSC Form 44</t>
-  </si>
-  <si>
-    <t>Ionizing Radiation Source Data Sheet-Space Flight
-Hardware and Applications</t>
-  </si>
-  <si>
-    <t>ISS_OE_851</t>
-  </si>
-  <si>
-    <t>Unique Hazard Report Form (DRD only)</t>
-  </si>
-  <si>
-    <t>ISS_OE_1298</t>
-  </si>
-  <si>
-    <t>Standard Hazard Report (DRD only)</t>
-  </si>
-  <si>
-    <t>ISS_Biosafety_713
-/ISS_OE_713</t>
-  </si>
-  <si>
-    <t>Inflight Biohazardous Materials Approval Form</t>
-  </si>
-  <si>
-    <t>P32928-103</t>
-  </si>
-  <si>
-    <t>Requirements for International Partner Cargoes
-transported on Russian Progress and Soyuz Vehicles</t>
-  </si>
-  <si>
-    <t>P32958-106</t>
-  </si>
-  <si>
-    <t>ISS Technical Requirements for Hardware to be Stored
-or Operated on the ISS Russian Segment</t>
-  </si>
-  <si>
-    <t>JSC 27472</t>
-  </si>
-  <si>
-    <t>rev. C</t>
-  </si>
-  <si>
-    <t>Requirements for Submission of Data needed for
-Toxicological Assessment of chemicals to be flown on
-manned Spacecraft</t>
-  </si>
-  <si>
-    <t>ISS_OE_Bio_ECLSS_T
-ox_Submittal</t>
-  </si>
-  <si>
-    <t>Hazardous Material Summary Table</t>
-  </si>
-  <si>
-    <t>ESA-ISS-COL-SECRS-0002</t>
-  </si>
-  <si>
-    <t>Security Requirements for LAN Connected Payloads</t>
-  </si>
-  <si>
-    <t>SSP 50989</t>
-  </si>
-  <si>
-    <t>ISS IT Security Policy for onboard Systems</t>
-  </si>
-  <si>
-    <t>ESSB-ST-E-008</t>
-  </si>
-  <si>
-    <t>Secure Software Engineering Standard (04 July 2016)</t>
-  </si>
-  <si>
-    <t>Rev. 1</t>
-  </si>
-  <si>
-    <t>System engineering general requirements (15 February 2017)</t>
-  </si>
-  <si>
-    <t>ECSS-E-ST-10</t>
+    <t>es</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -11520,15 +10576,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -11538,11 +10587,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="22"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -11555,10 +10599,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -11584,10 +10627,9 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Schlecht" xfId="2" builtinId="27"/>
+  <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2" xfId="1" xr:uid="{13AC667A-421C-422C-A418-8593B8FE388E}"/>
   </cellStyles>
@@ -11911,6 +10953,7 @@
     <col min="5" max="5" width="58.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="4.77734375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="50" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -11935,6 +10978,7 @@
       <c r="G1" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="H1" s="6"/>
     </row>
     <row r="2" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -12056,6 +11100,7 @@
       <c r="G6" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="H6" s="6"/>
     </row>
     <row r="7" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
@@ -12102,6 +11147,7 @@
       <c r="G8" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="H8" s="6"/>
     </row>
     <row r="9" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
@@ -12194,6 +11240,7 @@
       <c r="G12" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="H12" s="6"/>
     </row>
     <row r="13" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
@@ -12287,7 +11334,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>23</v>
       </c>
@@ -12309,8 +11356,9 @@
       <c r="G17" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="H17" s="6"/>
+    </row>
+    <row r="18" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>3</v>
       </c>
@@ -12333,7 +11381,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>25</v>
       </c>
@@ -12355,8 +11403,9 @@
       <c r="G19" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="H19" s="6"/>
+    </row>
+    <row r="20" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>3</v>
       </c>
@@ -12379,7 +11428,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>29</v>
       </c>
@@ -12401,8 +11450,9 @@
       <c r="G21" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="H21" s="6"/>
+    </row>
+    <row r="22" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>3</v>
       </c>
@@ -12425,7 +11475,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>7</v>
       </c>
@@ -12448,7 +11498,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>9</v>
       </c>
@@ -12471,7 +11521,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -12494,7 +11544,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>31</v>
       </c>
@@ -12517,7 +11567,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>33</v>
       </c>
@@ -12540,7 +11590,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>35</v>
       </c>
@@ -12563,7 +11613,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>37</v>
       </c>
@@ -12586,7 +11636,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>39</v>
       </c>
@@ -12609,7 +11659,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>3</v>
       </c>
@@ -12632,7 +11682,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>7</v>
       </c>
@@ -85313,7 +84363,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="C1:H1" xr:uid="{8A3BDAC9-4A16-4B5D-8A8F-A759210B771D}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -87087,7 +86137,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0DB6761-418B-4A4C-A696-A4E454C17842}">
-  <dimension ref="A1:E147"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" style="8"/>
@@ -87116,1888 +86166,20 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
-        <v>9</v>
+      <c r="A2" s="9" t="s">
+        <v>3399</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>3398</v>
+        <v>3392</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>3396</v>
       </c>
+      <c r="D2" s="8" t="s">
+        <v>3397</v>
+      </c>
       <c r="E2" s="8" t="s">
-        <v>3399</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>3400</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>3397</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>3401</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>3402</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>3403</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>3404</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>3405</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>3406</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>3407</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>3408</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>3409</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>3410</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>3411</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>3412</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>3413</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>3397</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>3414</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>3415</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>3397</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>3416</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>3417</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>3418</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>3419</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>3420</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>3421</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>3422</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>3403</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>3423</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>3424</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>3425</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>3426</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>3397</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>3427</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>3428</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>3397</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>3429</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>3430</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>3431</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>3432</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>3433</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>3434</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>3397</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>3435</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>3436</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>3403</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>3437</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>3438</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D21" s="8" t="s">
-        <v>3403</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>3439</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>3440</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>3441</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>3442</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E23" s="8" t="s">
-        <v>3443</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>3444</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D24" s="8" t="s">
-        <v>3397</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>3445</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>3446</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>3397</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>3447</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>3448</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>3449</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>3450</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>3451</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>3452</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>3397</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>3453</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>3454</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>3455</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>3456</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E30" s="8" t="s">
-        <v>3457</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>3458</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E31" s="8" t="s">
-        <v>3459</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A32" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>3460</v>
-      </c>
-      <c r="C32" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E32" s="8" t="s">
-        <v>3461</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>3462</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D33" s="8" t="s">
-        <v>3397</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>3463</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>3464</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E34" s="8" t="s">
-        <v>3465</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>3466</v>
-      </c>
-      <c r="C35" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>3467</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="B36" s="8" t="s">
-        <v>3468</v>
-      </c>
-      <c r="C36" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E36" s="8" t="s">
-        <v>3469</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A37" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="B37" s="8" t="s">
-        <v>3470</v>
-      </c>
-      <c r="C37" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>3471</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A38" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="B38" s="8" t="s">
-        <v>3472</v>
-      </c>
-      <c r="C38" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E38" s="8" t="s">
-        <v>3473</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A39" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="B39" s="8" t="s">
-        <v>3474</v>
-      </c>
-      <c r="C39" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E39" s="8" t="s">
-        <v>3475</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A40" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="B40" s="8" t="s">
-        <v>3476</v>
-      </c>
-      <c r="C40" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E40" s="8" t="s">
-        <v>3477</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A41" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="B41" s="8" t="s">
-        <v>3478</v>
-      </c>
-      <c r="C41" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E41" s="8" t="s">
-        <v>3479</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A42" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="B42" s="8" t="s">
-        <v>3480</v>
-      </c>
-      <c r="C42" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E42" s="8" t="s">
-        <v>3481</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A43" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>3482</v>
-      </c>
-      <c r="C43" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E43" s="8" t="s">
-        <v>3483</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A44" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="B44" s="8" t="s">
-        <v>3484</v>
-      </c>
-      <c r="C44" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E44" s="8" t="s">
-        <v>3485</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A45" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="B45" s="8" t="s">
-        <v>3486</v>
-      </c>
-      <c r="C45" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D45" s="8" t="s">
-        <v>3397</v>
-      </c>
-      <c r="E45" s="8" t="s">
-        <v>3487</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A46" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="B46" s="8" t="s">
-        <v>3488</v>
-      </c>
-      <c r="C46" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E46" s="8" t="s">
-        <v>3489</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A47" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="B47" s="8" t="s">
-        <v>3490</v>
-      </c>
-      <c r="C47" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E47" s="8" t="s">
-        <v>3491</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A48" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="B48" s="8" t="s">
-        <v>3492</v>
-      </c>
-      <c r="C48" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E48" s="8" t="s">
-        <v>3493</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A49" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="B49" s="8" t="s">
-        <v>3494</v>
-      </c>
-      <c r="C49" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E49" s="8" t="s">
-        <v>3495</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A50" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="B50" s="8" t="s">
-        <v>3496</v>
-      </c>
-      <c r="C50" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D50" s="8" t="s">
-        <v>3497</v>
-      </c>
-      <c r="E50" s="8" t="s">
-        <v>3498</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A51" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="B51" s="8" t="s">
-        <v>3499</v>
-      </c>
-      <c r="C51" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E51" s="8" t="s">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A52" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="B52" s="8" t="s">
-        <v>3501</v>
-      </c>
-      <c r="C52" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E52" s="8" t="s">
-        <v>3502</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A53" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="B53" s="8" t="s">
-        <v>3503</v>
-      </c>
-      <c r="C53" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E53" s="8" t="s">
-        <v>3504</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A54" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="B54" s="8" t="s">
-        <v>3505</v>
-      </c>
-      <c r="C54" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E54" s="8" t="s">
-        <v>3506</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A55" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="B55" s="8" t="s">
-        <v>3507</v>
-      </c>
-      <c r="C55" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E55" s="8" t="s">
-        <v>3508</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A56" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="B56" s="8" t="s">
-        <v>3509</v>
-      </c>
-      <c r="C56" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E56" s="8" t="s">
-        <v>3510</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A57" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="B57" s="8" t="s">
-        <v>3511</v>
-      </c>
-      <c r="C57" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D57" s="8" t="s">
-        <v>3512</v>
-      </c>
-      <c r="E57" s="8" t="s">
-        <v>3513</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A58" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="B58" s="8" t="s">
-        <v>3514</v>
-      </c>
-      <c r="C58" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E58" s="8" t="s">
-        <v>3515</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A59" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="B59" s="8" t="s">
-        <v>3392</v>
-      </c>
-      <c r="C59" s="8" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D59" s="8" t="s">
-        <v>3397</v>
-      </c>
-      <c r="E59" s="8" t="s">
-        <v>3516</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A60" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="B60" s="8" t="s">
-        <v>3517</v>
-      </c>
-      <c r="E60" s="8" t="s">
-        <v>3518</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A61" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="B61" s="8" t="s">
-        <v>3519</v>
-      </c>
-      <c r="E61" s="8" t="s">
-        <v>3520</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A62" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="B62" s="8" t="s">
-        <v>3521</v>
-      </c>
-      <c r="E62" s="8" t="s">
-        <v>3522</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A63" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="B63" s="8" t="s">
-        <v>3523</v>
-      </c>
-      <c r="E63" s="8" t="s">
-        <v>3524</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A64" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="B64" s="8" t="s">
-        <v>3525</v>
-      </c>
-      <c r="E64" s="8" t="s">
-        <v>3526</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A65" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="B65" s="8" t="s">
-        <v>3527</v>
-      </c>
-      <c r="D65" s="8" t="s">
-        <v>3528</v>
-      </c>
-      <c r="E65" s="8" t="s">
-        <v>3529</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A66" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="B66" s="8" t="s">
-        <v>3530</v>
-      </c>
-      <c r="E66" s="8" t="s">
-        <v>3531</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A67" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="B67" s="8" t="s">
-        <v>3532</v>
-      </c>
-      <c r="E67" s="8" t="s">
-        <v>3533</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A68" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="B68" s="8" t="s">
-        <v>3534</v>
-      </c>
-      <c r="E68" s="8" t="s">
-        <v>3535</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A69" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="B69" s="8" t="s">
-        <v>3536</v>
-      </c>
-      <c r="E69" s="8" t="s">
-        <v>3537</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A70" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="B70" s="8" t="s">
-        <v>3538</v>
-      </c>
-      <c r="E70" s="8" t="s">
-        <v>3539</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A71" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="B71" s="8" t="s">
-        <v>3540</v>
-      </c>
-      <c r="E71" s="8" t="s">
-        <v>3541</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A72" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="B72" s="8" t="s">
-        <v>3542</v>
-      </c>
-      <c r="E72" s="8" t="s">
-        <v>3543</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A73" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="B73" s="8" t="s">
-        <v>3544</v>
-      </c>
-      <c r="E73" s="8" t="s">
-        <v>3545</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A74" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="B74" s="8" t="s">
-        <v>3546</v>
-      </c>
-      <c r="D74" s="8" t="s">
-        <v>3547</v>
-      </c>
-      <c r="E74" s="8" t="s">
-        <v>3548</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A75" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="B75" s="8" t="s">
-        <v>3549</v>
-      </c>
-      <c r="E75" s="8" t="s">
-        <v>3550</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A76" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="B76" s="8" t="s">
-        <v>3551</v>
-      </c>
-      <c r="E76" s="8" t="s">
-        <v>3552</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A77" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="B77" s="8" t="s">
-        <v>3553</v>
-      </c>
-      <c r="E77" s="8" t="s">
-        <v>3554</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A78" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="B78" s="8" t="s">
-        <v>3555</v>
-      </c>
-      <c r="E78" s="8" t="s">
-        <v>3556</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A79" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="B79" s="8" t="s">
-        <v>3557</v>
-      </c>
-      <c r="E79" s="8" t="s">
-        <v>3558</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A80" s="8" t="s">
-        <v>160</v>
-      </c>
-      <c r="B80" s="8" t="s">
-        <v>3559</v>
-      </c>
-      <c r="E80" s="8" t="s">
-        <v>3560</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A81" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="B81" s="8" t="s">
-        <v>3561</v>
-      </c>
-      <c r="E81" s="8" t="s">
-        <v>3562</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A82" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="B82" s="8" t="s">
-        <v>3563</v>
-      </c>
-      <c r="E82" s="8" t="s">
-        <v>3564</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A83" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="B83" s="8" t="s">
-        <v>3565</v>
-      </c>
-      <c r="D83" s="8" t="s">
-        <v>3566</v>
-      </c>
-      <c r="E83" s="8" t="s">
-        <v>3567</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A84" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="B84" s="8" t="s">
-        <v>3568</v>
-      </c>
-      <c r="E84" s="8" t="s">
-        <v>3569</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A85" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="B85" s="8" t="s">
-        <v>3570</v>
-      </c>
-      <c r="E85" s="8" t="s">
-        <v>3571</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A86" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="B86" s="8" t="s">
-        <v>3572</v>
-      </c>
-      <c r="E86" s="8" t="s">
-        <v>3573</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A87" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="B87" s="8" t="s">
-        <v>3574</v>
-      </c>
-      <c r="E87" s="8" t="s">
-        <v>3575</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A88" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="B88" s="8" t="s">
-        <v>3576</v>
-      </c>
-      <c r="E88" s="8" t="s">
-        <v>3577</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A89" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="B89" s="8" t="s">
-        <v>3580</v>
-      </c>
-      <c r="E89" s="8" t="s">
-        <v>3578</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A90" s="8" t="s">
-        <v>172</v>
-      </c>
-      <c r="B90" s="8" t="s">
-        <v>3579</v>
-      </c>
-      <c r="E90" s="8" t="s">
-        <v>3581</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A91" s="8" t="s">
-        <v>173</v>
-      </c>
-      <c r="B91" s="8" t="s">
-        <v>3582</v>
-      </c>
-      <c r="E91" s="8" t="s">
-        <v>3583</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A92" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="B92" s="8" t="s">
-        <v>3584</v>
-      </c>
-      <c r="E92" s="8" t="s">
-        <v>3585</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A93" s="8" t="s">
-        <v>175</v>
-      </c>
-      <c r="B93" s="8" t="s">
-        <v>3586</v>
-      </c>
-      <c r="E93" s="8" t="s">
-        <v>3588</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A94" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="B94" s="8" t="s">
-        <v>3587</v>
-      </c>
-      <c r="E94" s="8" t="s">
-        <v>3589</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A95" s="8" t="s">
-        <v>178</v>
-      </c>
-      <c r="B95" s="8" t="s">
-        <v>3590</v>
-      </c>
-      <c r="E95" s="8" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A96" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="B96" s="8" t="s">
-        <v>3591</v>
-      </c>
-      <c r="E96" s="8" t="s">
-        <v>3592</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A97" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="B97" s="8" t="s">
-        <v>3593</v>
-      </c>
-      <c r="E97" s="8" t="s">
-        <v>3594</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A98" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="B98" s="8" t="s">
-        <v>3595</v>
-      </c>
-      <c r="E98" s="8" t="s">
-        <v>3596</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A99" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="B99" s="8" t="s">
-        <v>3597</v>
-      </c>
-      <c r="E99" s="8" t="s">
-        <v>3598</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A100" s="8" t="s">
-        <v>186</v>
-      </c>
-      <c r="B100" s="8" t="s">
-        <v>3599</v>
-      </c>
-      <c r="E100" s="8" t="s">
-        <v>3600</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A101" s="8" t="s">
-        <v>187</v>
-      </c>
-      <c r="B101" s="8" t="s">
-        <v>3601</v>
-      </c>
-      <c r="E101" s="8" t="s">
-        <v>3602</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A102" s="8" t="s">
-        <v>188</v>
-      </c>
-      <c r="B102" s="8" t="s">
-        <v>3603</v>
-      </c>
-      <c r="E102" s="8" t="s">
-        <v>3604</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A103" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="B103" s="8" t="s">
-        <v>3605</v>
-      </c>
-      <c r="E103" s="8" t="s">
-        <v>3606</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A104" s="8" t="s">
-        <v>191</v>
-      </c>
-      <c r="B104" s="8" t="s">
-        <v>3607</v>
-      </c>
-      <c r="E104" s="8" t="s">
-        <v>3608</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A105" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="B105" s="8" t="s">
-        <v>3609</v>
-      </c>
-      <c r="E105" s="8" t="s">
-        <v>3610</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A106" s="8" t="s">
-        <v>193</v>
-      </c>
-      <c r="B106" s="8" t="s">
-        <v>3611</v>
-      </c>
-      <c r="E106" s="8" t="s">
-        <v>3612</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A107" s="8" t="s">
-        <v>195</v>
-      </c>
-      <c r="B107" s="8" t="s">
-        <v>3613</v>
-      </c>
-      <c r="E107" s="8" t="s">
-        <v>3614</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A108" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="B108" s="8" t="s">
-        <v>3615</v>
-      </c>
-      <c r="E108" s="8" t="s">
-        <v>3616</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A109" s="8" t="s">
-        <v>199</v>
-      </c>
-      <c r="B109" s="8" t="s">
-        <v>3617</v>
-      </c>
-      <c r="D109" s="8" t="s">
-        <v>3566</v>
-      </c>
-      <c r="E109" s="8" t="s">
-        <v>3618</v>
-      </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A110" s="8" t="s">
-        <v>200</v>
-      </c>
-      <c r="B110" s="8" t="s">
-        <v>3619</v>
-      </c>
-      <c r="D110" s="8" t="s">
-        <v>3566</v>
-      </c>
-      <c r="E110" s="8" t="s">
-        <v>3620</v>
-      </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A111" s="8" t="s">
-        <v>201</v>
-      </c>
-      <c r="B111" s="8" t="s">
-        <v>3621</v>
-      </c>
-      <c r="E111" s="8" t="s">
-        <v>3622</v>
-      </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A112" s="8" t="s">
-        <v>202</v>
-      </c>
-      <c r="B112" s="8" t="s">
-        <v>3623</v>
-      </c>
-      <c r="E112" s="8" t="s">
-        <v>3624</v>
-      </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A113" s="8" t="s">
-        <v>204</v>
-      </c>
-      <c r="B113" s="8" t="s">
-        <v>3625</v>
-      </c>
-      <c r="E113" s="8" t="s">
-        <v>3628</v>
-      </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A114" s="8" t="s">
-        <v>205</v>
-      </c>
-      <c r="B114" s="8" t="s">
-        <v>3626</v>
-      </c>
-      <c r="E114" s="8" t="s">
-        <v>3627</v>
-      </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A115" s="8" t="s">
-        <v>206</v>
-      </c>
-      <c r="B115" s="8" t="s">
-        <v>3629</v>
-      </c>
-      <c r="E115" s="8" t="s">
-        <v>3630</v>
-      </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A116" s="8" t="s">
-        <v>207</v>
-      </c>
-      <c r="E116" s="8" t="s">
-        <v>3631</v>
-      </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A117" s="8" t="s">
-        <v>208</v>
-      </c>
-      <c r="B117" s="8" t="s">
-        <v>3632</v>
-      </c>
-      <c r="D117" s="8" t="s">
-        <v>3633</v>
-      </c>
-      <c r="E117" s="8" t="s">
-        <v>3634</v>
-      </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A118" s="8" t="s">
-        <v>209</v>
-      </c>
-      <c r="B118" s="8" t="s">
-        <v>3635</v>
-      </c>
-      <c r="D118" s="8" t="s">
-        <v>3633</v>
-      </c>
-      <c r="E118" s="8" t="s">
-        <v>3636</v>
-      </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A119" s="8" t="s">
-        <v>211</v>
-      </c>
-      <c r="B119" s="8" t="s">
-        <v>3637</v>
-      </c>
-      <c r="E119" s="8" t="s">
-        <v>3638</v>
-      </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A120" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="B120" s="8" t="s">
-        <v>3639</v>
-      </c>
-      <c r="D120" s="8" t="s">
-        <v>3640</v>
-      </c>
-      <c r="E120" s="8" t="s">
-        <v>3641</v>
-      </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A121" s="8" t="s">
-        <v>214</v>
-      </c>
-      <c r="B121" s="8" t="s">
-        <v>3642</v>
-      </c>
-      <c r="D121" s="8" t="s">
-        <v>3643</v>
-      </c>
-      <c r="E121" s="8" t="s">
-        <v>3644</v>
-      </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A122" s="8" t="s">
-        <v>215</v>
-      </c>
-      <c r="B122" s="8" t="s">
-        <v>3645</v>
-      </c>
-      <c r="D122" s="8" t="s">
-        <v>3643</v>
-      </c>
-      <c r="E122" s="8" t="s">
-        <v>3646</v>
-      </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A123" s="8" t="s">
-        <v>217</v>
-      </c>
-      <c r="B123" s="8" t="s">
-        <v>3647</v>
-      </c>
-      <c r="D123" s="8" t="s">
-        <v>3643</v>
-      </c>
-      <c r="E123" s="8" t="s">
-        <v>3648</v>
-      </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A124" s="8" t="s">
-        <v>218</v>
-      </c>
-      <c r="B124" s="8" t="s">
-        <v>3649</v>
-      </c>
-      <c r="D124" s="8" t="s">
-        <v>3650</v>
-      </c>
-      <c r="E124" s="8" t="s">
-        <v>3651</v>
-      </c>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A125" s="8" t="s">
-        <v>219</v>
-      </c>
-      <c r="B125" s="8" t="s">
-        <v>3652</v>
-      </c>
-      <c r="D125" s="8" t="s">
-        <v>3653</v>
-      </c>
-      <c r="E125" s="8" t="s">
-        <v>3654</v>
-      </c>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A126" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="B126" s="8" t="s">
-        <v>3655</v>
-      </c>
-      <c r="D126" s="8" t="s">
-        <v>3656</v>
-      </c>
-      <c r="E126" s="8" t="s">
-        <v>3657</v>
-      </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A127" s="8" t="s">
-        <v>222</v>
-      </c>
-      <c r="B127" s="8" t="s">
-        <v>3658</v>
-      </c>
-      <c r="E127" s="8" t="s">
-        <v>3659</v>
-      </c>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A128" s="8" t="s">
-        <v>224</v>
-      </c>
-      <c r="B128" s="8" t="s">
-        <v>3662</v>
-      </c>
-      <c r="E128" s="8" t="s">
-        <v>3663</v>
-      </c>
-    </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A129" s="8" t="s">
-        <v>226</v>
-      </c>
-      <c r="B129" s="8" t="s">
-        <v>3660</v>
-      </c>
-      <c r="E129" s="8" t="s">
-        <v>3661</v>
-      </c>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A130" s="8" t="s">
-        <v>227</v>
-      </c>
-      <c r="B130" s="8" t="s">
-        <v>3664</v>
-      </c>
-      <c r="E130" s="8" t="s">
-        <v>3665</v>
-      </c>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A131" s="8" t="s">
-        <v>229</v>
-      </c>
-      <c r="B131" s="8" t="s">
-        <v>3666</v>
-      </c>
-      <c r="E131" s="8" t="s">
-        <v>3667</v>
-      </c>
-    </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A132" s="8" t="s">
-        <v>231</v>
-      </c>
-      <c r="B132" s="8" t="s">
-        <v>3668</v>
-      </c>
-      <c r="E132" s="8" t="s">
-        <v>3669</v>
-      </c>
-    </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A133" s="8" t="s">
-        <v>232</v>
-      </c>
-      <c r="B133" s="8" t="s">
-        <v>3670</v>
-      </c>
-      <c r="E133" s="8" t="s">
-        <v>3671</v>
-      </c>
-    </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A134" s="8" t="s">
-        <v>234</v>
-      </c>
-      <c r="B134" s="8" t="s">
-        <v>3672</v>
-      </c>
-      <c r="E134" s="8" t="s">
-        <v>3673</v>
-      </c>
-    </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A135" s="8" t="s">
-        <v>235</v>
-      </c>
-      <c r="B135" s="8" t="s">
-        <v>3674</v>
-      </c>
-      <c r="E135" s="8" t="s">
-        <v>3675</v>
-      </c>
-    </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A136" s="8" t="s">
-        <v>236</v>
-      </c>
-      <c r="B136" s="8" t="s">
-        <v>3676</v>
-      </c>
-      <c r="E136" s="8" t="s">
-        <v>3677</v>
-      </c>
-    </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A137" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="B137" s="8" t="s">
-        <v>3678</v>
-      </c>
-      <c r="E137" s="8" t="s">
-        <v>3679</v>
-      </c>
-    </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A138" s="8" t="s">
-        <v>239</v>
-      </c>
-      <c r="B138" s="8" t="s">
-        <v>3680</v>
-      </c>
-      <c r="E138" s="8" t="s">
-        <v>3681</v>
-      </c>
-    </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A139" s="8" t="s">
-        <v>240</v>
-      </c>
-      <c r="B139" s="8" t="s">
-        <v>3682</v>
-      </c>
-      <c r="E139" s="8" t="s">
-        <v>3683</v>
-      </c>
-    </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A140" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="B140" s="8" t="s">
-        <v>3684</v>
-      </c>
-      <c r="E140" s="8" t="s">
-        <v>3685</v>
-      </c>
-    </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A141" s="8" t="s">
-        <v>242</v>
-      </c>
-      <c r="B141" s="8" t="s">
-        <v>3686</v>
-      </c>
-      <c r="E141" s="8" t="s">
-        <v>3687</v>
-      </c>
-    </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A142" s="8" t="s">
-        <v>243</v>
-      </c>
-      <c r="B142" s="8" t="s">
-        <v>3688</v>
-      </c>
-      <c r="D142" s="8" t="s">
-        <v>3689</v>
-      </c>
-      <c r="E142" s="8" t="s">
-        <v>3690</v>
-      </c>
-    </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A143" s="8" t="s">
-        <v>245</v>
-      </c>
-      <c r="B143" s="8" t="s">
-        <v>3691</v>
-      </c>
-      <c r="E143" s="8" t="s">
-        <v>3692</v>
-      </c>
-    </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A144" s="8" t="s">
-        <v>246</v>
-      </c>
-      <c r="B144" s="8" t="s">
-        <v>3693</v>
-      </c>
-      <c r="E144" s="8" t="s">
-        <v>3694</v>
-      </c>
-    </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A145" s="8" t="s">
-        <v>248</v>
-      </c>
-      <c r="B145" s="8" t="s">
-        <v>3695</v>
-      </c>
-      <c r="E145" s="8" t="s">
-        <v>3696</v>
-      </c>
-    </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A146" s="8" t="s">
-        <v>249</v>
-      </c>
-      <c r="B146" s="8" t="s">
-        <v>3697</v>
-      </c>
-      <c r="E146" s="8" t="s">
-        <v>3698</v>
-      </c>
-    </row>
-    <row r="147" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="9" t="s">
-        <v>250</v>
-      </c>
-      <c r="B147" s="9" t="s">
-        <v>3701</v>
-      </c>
-      <c r="C147" s="9" t="s">
-        <v>3396</v>
-      </c>
-      <c r="D147" s="9" t="s">
-        <v>3699</v>
-      </c>
-      <c r="E147" s="9" t="s">
-        <v>3700</v>
+        <v>3398</v>
       </c>
     </row>
   </sheetData>

</xml_diff>